<commit_message>
Mise à jour Patient et Practitioner (#34)
* update patient and practitioner

* update 924ba600e5bb1b39c1013f3a1b541e3b3cc4f640
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-composition-document.xlsx
+++ b/main/ig/StructureDefinition-fr-composition-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-21T08:14:34+00:00</t>
+    <t>2025-10-21T15:23:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1661,7 +1661,7 @@
     <t>Auteur du document</t>
   </si>
   <si>
-    <t>author permet d’enregistrer un auteur du document. Un document peut avoir un ou plusieurs auteurs.</t>
+    <t>author permet d’enregistrer un auteur du document. Un document peut avoir un ou plusieurs auteurs. Un professionnel de santé auteur d'un document est toujours dans une situation d'exercice donnée (FrPractitionerRoleDocument).</t>
   </si>
   <si>
     <t>Identifies who is responsible for the content.</t>

</xml_diff>